<commit_message>
Changed base URL for artifacts, changed referralType (CodeableConcept) parameter to isProviderReferral (boolean) for the  operation.
</commit_message>
<xml_diff>
--- a/CodeSystem-ACCESSAlignmentResultCS.xlsx
+++ b/CodeSystem-ACCESSAlignmentResultCS.xlsx
@@ -24,13 +24,13 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://globalalliantinc.com/access/CodeSystem/ACCESSAlignmentResultCS</t>
+    <t>https://dsacms.github.io/cmmi-access-model/CodeSystem/ACCESSAlignmentResultCS</t>
   </si>
   <si>
     <t>Version</t>
   </si>
   <si>
-    <t>0.9.0</t>
+    <t>0.9.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-06T16:03:26-05:00</t>
+    <t>2026-03-12T23:55:37-07:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Updated ACCESS Model IG and ACCESS Model Operations Manual to v0.9.6.
</commit_message>
<xml_diff>
--- a/CodeSystem-ACCESSAlignmentResultCS.xlsx
+++ b/CodeSystem-ACCESSAlignmentResultCS.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.9.1</t>
+    <t>0.9.6</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-12T23:55:37-07:00</t>
+    <t>2026-04-24T13:45:33-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -168,7 +168,7 @@
     <t>Not aligned - already aligned to another participant in the track</t>
   </si>
   <si>
-    <t>The patient is technically eligible, but is already aligned to another participant and receiving services under the ACCESS Model in the same track. A patient can only be aligned to one participant in each track. If a switch consent attestation is submitted, but the patient is still within the 3-month lock-in period, this response will be received.</t>
+    <t>The patient is technically eligible, but is already aligned to another participant and receiving services under the ACCESS Model in the same track. A patient can only be aligned to one participant in each track. If a switch consent attestation is submitted, but the patient is still within the 90-day lock-in period, this response will be received.</t>
   </si>
   <si>
     <t>not-aligned-not-medicare</t>
@@ -204,7 +204,7 @@
     <t>Aligned and switch approved</t>
   </si>
   <si>
-    <t>The request to switch the patient's alignment from a different participant after the 3-month lock in period is accepted and the patient is considered switched and now re-aligned.</t>
+    <t>The request to switch the patient's alignment from a different participant after the 90-day lock in period is accepted and the patient is considered switched and now re-aligned.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Added ACCESS Model IG 0.9.8 files.
</commit_message>
<xml_diff>
--- a/CodeSystem-ACCESSAlignmentResultCS.xlsx
+++ b/CodeSystem-ACCESSAlignmentResultCS.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="73">
   <si>
     <t>Property</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.9.6</t>
+    <t>0.9.8</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-24T13:45:33-04:00</t>
+    <t>2026-05-18T15:59:44-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -126,7 +126,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>7</t>
+    <t>10</t>
   </si>
   <si>
     <t>Level</t>
@@ -153,6 +153,15 @@
     <t>Patient is eligible and has been aligned so the participant can now begin providing services to the patient under the ACCESS Model.</t>
   </si>
   <si>
+    <t>aligned-switch-approved</t>
+  </si>
+  <si>
+    <t>Aligned and switch approved</t>
+  </si>
+  <si>
+    <t>The request to switch the patient's alignment from a different participant after the 90-day lock in period is accepted and the patient is considered switched and now re-aligned.</t>
+  </si>
+  <si>
     <t>not-aligned-control-group</t>
   </si>
   <si>
@@ -198,13 +207,31 @@
     <t>The patient does not have a treating diagnosis that qualifies them for service in the track indicated and therefore cannot get services under the ACCESS Model.</t>
   </si>
   <si>
-    <t>aligned-switch-approved</t>
-  </si>
-  <si>
-    <t>Aligned and switch approved</t>
-  </si>
-  <si>
-    <t>The request to switch the patient's alignment from a different participant after the 90-day lock in period is accepted and the patient is considered switched and now re-aligned.</t>
+    <t>not-aligned-clinical-exclusion</t>
+  </si>
+  <si>
+    <t>Not aligned - clinical exclusion</t>
+  </si>
+  <si>
+    <t>The patient has a clinical exclusion that prevents them from receiving services under the ACCESS Model.</t>
+  </si>
+  <si>
+    <t>not-aligned-mismatch</t>
+  </si>
+  <si>
+    <t>Not aligned - mismatch</t>
+  </si>
+  <si>
+    <t>The patient information provided does not match the patient information on record.</t>
+  </si>
+  <si>
+    <t>not-aligned-no-switch-attestation</t>
+  </si>
+  <si>
+    <t>Not aligned - no switch attestation</t>
+  </si>
+  <si>
+    <t>Participant switch request did not include switch consent attestation.</t>
   </si>
 </sst>
 </file>
@@ -516,7 +543,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -631,6 +658,48 @@
         <v>63</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B9" t="s" s="2">
+        <v>64</v>
+      </c>
+      <c r="C9" t="s" s="2">
+        <v>65</v>
+      </c>
+      <c r="D9" t="s" s="2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B10" t="s" s="2">
+        <v>67</v>
+      </c>
+      <c r="C10" t="s" s="2">
+        <v>68</v>
+      </c>
+      <c r="D10" t="s" s="2">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B11" t="s" s="2">
+        <v>70</v>
+      </c>
+      <c r="C11" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="D11" t="s" s="2">
+        <v>72</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated to ACCESS Model IG 0.9.11 and Operations Manual 0.9.11.
</commit_message>
<xml_diff>
--- a/CodeSystem-ACCESSAlignmentResultCS.xlsx
+++ b/CodeSystem-ACCESSAlignmentResultCS.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.9.8</t>
+    <t>0.9.11</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-20T09:30:43-04:00</t>
+    <t>2026-06-04T22:54:52-04:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Updated IG to v0.9.12.
</commit_message>
<xml_diff>
--- a/CodeSystem-ACCESSAlignmentResultCS.xlsx
+++ b/CodeSystem-ACCESSAlignmentResultCS.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.9.11</t>
+    <t>0.9.12</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-04T23:05:21-04:00</t>
+    <t>2026-06-10T23:08:55-04:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>